<commit_message>
Problem solve confidence intervals
</commit_message>
<xml_diff>
--- a/data/ModelResults.xlsx
+++ b/data/ModelResults.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://michiganstate-my.sharepoint.com/personal/buysseso_msu_edu/Documents/Arabidopsis/Swe_Italy/R_scripts/SW_IT_PopDiffPlasticity/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1004" documentId="13_ncr:1_{AD4A5BE6-D9C1-414A-81C8-3A9C273D7774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C39365A8-E987-4FF2-BA00-A7F54868048B}"/>
+  <xr:revisionPtr revIDLastSave="1010" documentId="13_ncr:1_{AD4A5BE6-D9C1-414A-81C8-3A9C273D7774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3257DA11-BD6E-4106-98BA-D5927AD34A08}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{8A213037-8BA5-417B-A75A-3088B4717938}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{8A213037-8BA5-417B-A75A-3088B4717938}"/>
   </bookViews>
   <sheets>
     <sheet name="ModelResults" sheetId="1" r:id="rId1"/>
@@ -919,7 +919,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -974,6 +974,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -981,9 +984,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1025,6 +1025,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1401,24 +1402,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="40">
+      <c r="C1" s="41">
         <v>2021</v>
       </c>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="41"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="40">
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="41">
         <v>2022</v>
       </c>
-      <c r="K1" s="41"/>
-      <c r="L1" s="41"/>
-      <c r="M1" s="41"/>
-      <c r="N1" s="41"/>
-      <c r="O1" s="41"/>
-      <c r="P1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="43"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -1609,12 +1610,12 @@
       <c r="B6" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="43"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="43"/>
-      <c r="F6" s="43"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="43"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="40"/>
       <c r="I6" s="1"/>
       <c r="J6" s="1">
         <v>3.5658276954852297E-2</v>
@@ -1640,7 +1641,7 @@
       <c r="A7" s="36" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="10" t="s">
         <v>9</v>
       </c>
       <c r="C7" s="1">
@@ -1677,7 +1678,7 @@
       <c r="N7" s="1">
         <v>1.6096699122529901</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="57">
         <v>0.20766835063809</v>
       </c>
       <c r="P7" s="1"/>
@@ -1775,12 +1776,12 @@
       <c r="B10" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="43"/>
-      <c r="F10" s="43"/>
-      <c r="G10" s="43"/>
-      <c r="H10" s="43"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
+      <c r="G10" s="40"/>
+      <c r="H10" s="40"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1">
         <v>8.3492792785920695</v>
@@ -1907,12 +1908,12 @@
       <c r="B14" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="43"/>
-      <c r="D14" s="43"/>
-      <c r="E14" s="43"/>
-      <c r="F14" s="43"/>
-      <c r="G14" s="43"/>
-      <c r="H14" s="43"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="40"/>
+      <c r="E14" s="40"/>
+      <c r="F14" s="40"/>
+      <c r="G14" s="40"/>
+      <c r="H14" s="40"/>
       <c r="I14" s="1"/>
       <c r="J14" s="39"/>
       <c r="K14" s="39"/>
@@ -2026,12 +2027,12 @@
       <c r="B18" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C18" s="43"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="43"/>
-      <c r="F18" s="43"/>
-      <c r="G18" s="43"/>
-      <c r="H18" s="43"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="40"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="40"/>
       <c r="I18" s="1"/>
       <c r="J18" s="39"/>
       <c r="K18" s="39"/>
@@ -2170,7 +2171,7 @@
       <c r="N21" s="1">
         <v>3.5502596702509801</v>
       </c>
-      <c r="O21" s="2">
+      <c r="O21" s="3">
         <v>6.2255752292747699E-2</v>
       </c>
       <c r="P21" s="1"/>
@@ -2180,12 +2181,12 @@
       <c r="B22" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C22" s="43"/>
-      <c r="D22" s="43"/>
-      <c r="E22" s="43"/>
-      <c r="F22" s="43"/>
-      <c r="G22" s="43"/>
-      <c r="H22" s="43"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="40"/>
+      <c r="E22" s="40"/>
+      <c r="F22" s="40"/>
+      <c r="G22" s="40"/>
+      <c r="H22" s="40"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1">
         <v>5.2456643231190104E-3</v>
@@ -2346,12 +2347,12 @@
       <c r="B26" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C26" s="43"/>
-      <c r="D26" s="43"/>
-      <c r="E26" s="43"/>
-      <c r="F26" s="43"/>
-      <c r="G26" s="43"/>
-      <c r="H26" s="43"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="40"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="40"/>
+      <c r="G26" s="40"/>
+      <c r="H26" s="40"/>
       <c r="I26" s="1"/>
       <c r="J26" s="1">
         <v>7.5239018444935397E-3</v>
@@ -2512,12 +2513,12 @@
       <c r="B30" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C30" s="43"/>
-      <c r="D30" s="43"/>
-      <c r="E30" s="43"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="43"/>
-      <c r="H30" s="43"/>
+      <c r="C30" s="40"/>
+      <c r="D30" s="40"/>
+      <c r="E30" s="40"/>
+      <c r="F30" s="40"/>
+      <c r="G30" s="40"/>
+      <c r="H30" s="40"/>
       <c r="I30" s="1"/>
       <c r="J30" s="5">
         <v>7.2143853443936604E-6</v>
@@ -2678,12 +2679,12 @@
       <c r="B34" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C34" s="43"/>
-      <c r="D34" s="43"/>
-      <c r="E34" s="43"/>
-      <c r="F34" s="43"/>
-      <c r="G34" s="43"/>
-      <c r="H34" s="43"/>
+      <c r="C34" s="40"/>
+      <c r="D34" s="40"/>
+      <c r="E34" s="40"/>
+      <c r="F34" s="40"/>
+      <c r="G34" s="40"/>
+      <c r="H34" s="40"/>
       <c r="I34" s="1"/>
       <c r="J34" s="1">
         <v>0.34951867520347901</v>
@@ -2844,12 +2845,12 @@
       <c r="B38" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C38" s="43"/>
-      <c r="D38" s="43"/>
-      <c r="E38" s="43"/>
-      <c r="F38" s="43"/>
-      <c r="G38" s="43"/>
-      <c r="H38" s="43"/>
+      <c r="C38" s="40"/>
+      <c r="D38" s="40"/>
+      <c r="E38" s="40"/>
+      <c r="F38" s="40"/>
+      <c r="G38" s="40"/>
+      <c r="H38" s="40"/>
       <c r="I38" s="1"/>
       <c r="J38" s="1">
         <v>2.5021778012642701</v>
@@ -3010,12 +3011,12 @@
       <c r="B42" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C42" s="43"/>
-      <c r="D42" s="43"/>
-      <c r="E42" s="43"/>
-      <c r="F42" s="43"/>
-      <c r="G42" s="43"/>
-      <c r="H42" s="43"/>
+      <c r="C42" s="40"/>
+      <c r="D42" s="40"/>
+      <c r="E42" s="40"/>
+      <c r="F42" s="40"/>
+      <c r="G42" s="40"/>
+      <c r="H42" s="40"/>
       <c r="I42" s="1"/>
       <c r="J42" s="1">
         <v>4.9184876384352101E-2</v>
@@ -3176,12 +3177,12 @@
       <c r="B46" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C46" s="43"/>
-      <c r="D46" s="43"/>
-      <c r="E46" s="43"/>
-      <c r="F46" s="43"/>
-      <c r="G46" s="43"/>
-      <c r="H46" s="43"/>
+      <c r="C46" s="40"/>
+      <c r="D46" s="40"/>
+      <c r="E46" s="40"/>
+      <c r="F46" s="40"/>
+      <c r="G46" s="40"/>
+      <c r="H46" s="40"/>
       <c r="I46" s="1"/>
       <c r="J46" s="1">
         <v>3.6858467316493698E-2</v>
@@ -3342,12 +3343,12 @@
       <c r="B50" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C50" s="43"/>
-      <c r="D50" s="43"/>
-      <c r="E50" s="43"/>
-      <c r="F50" s="43"/>
-      <c r="G50" s="43"/>
-      <c r="H50" s="43"/>
+      <c r="C50" s="40"/>
+      <c r="D50" s="40"/>
+      <c r="E50" s="40"/>
+      <c r="F50" s="40"/>
+      <c r="G50" s="40"/>
+      <c r="H50" s="40"/>
       <c r="I50" s="1"/>
       <c r="J50" s="1">
         <v>3.4846897009296399E-3</v>
@@ -3642,12 +3643,12 @@
       <c r="B58" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C58" s="43"/>
-      <c r="D58" s="43"/>
-      <c r="E58" s="43"/>
-      <c r="F58" s="43"/>
-      <c r="G58" s="43"/>
-      <c r="H58" s="43"/>
+      <c r="C58" s="40"/>
+      <c r="D58" s="40"/>
+      <c r="E58" s="40"/>
+      <c r="F58" s="40"/>
+      <c r="G58" s="40"/>
+      <c r="H58" s="40"/>
       <c r="I58" s="1"/>
       <c r="J58" s="1">
         <v>1.0524858270047699</v>
@@ -3774,12 +3775,12 @@
       <c r="B62" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C62" s="43"/>
-      <c r="D62" s="43"/>
-      <c r="E62" s="43"/>
-      <c r="F62" s="43"/>
-      <c r="G62" s="43"/>
-      <c r="H62" s="43"/>
+      <c r="C62" s="40"/>
+      <c r="D62" s="40"/>
+      <c r="E62" s="40"/>
+      <c r="F62" s="40"/>
+      <c r="G62" s="40"/>
+      <c r="H62" s="40"/>
       <c r="I62" s="1"/>
       <c r="J62" s="39"/>
       <c r="K62" s="39"/>
@@ -4158,12 +4159,12 @@
       <c r="B74" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C74" s="43"/>
-      <c r="D74" s="43"/>
-      <c r="E74" s="43"/>
-      <c r="F74" s="43"/>
-      <c r="G74" s="43"/>
-      <c r="H74" s="43"/>
+      <c r="C74" s="40"/>
+      <c r="D74" s="40"/>
+      <c r="E74" s="40"/>
+      <c r="F74" s="40"/>
+      <c r="G74" s="40"/>
+      <c r="H74" s="40"/>
       <c r="I74" s="1"/>
       <c r="J74" s="39"/>
       <c r="K74" s="39"/>
@@ -4410,12 +4411,12 @@
       <c r="B82" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C82" s="43"/>
-      <c r="D82" s="43"/>
-      <c r="E82" s="43"/>
-      <c r="F82" s="43"/>
-      <c r="G82" s="43"/>
-      <c r="H82" s="43"/>
+      <c r="C82" s="40"/>
+      <c r="D82" s="40"/>
+      <c r="E82" s="40"/>
+      <c r="F82" s="40"/>
+      <c r="G82" s="40"/>
+      <c r="H82" s="40"/>
       <c r="I82" s="1"/>
       <c r="J82" s="39"/>
       <c r="K82" s="39"/>
@@ -4662,12 +4663,12 @@
       <c r="B90" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C90" s="43"/>
-      <c r="D90" s="43"/>
-      <c r="E90" s="43"/>
-      <c r="F90" s="43"/>
-      <c r="G90" s="43"/>
-      <c r="H90" s="43"/>
+      <c r="C90" s="40"/>
+      <c r="D90" s="40"/>
+      <c r="E90" s="40"/>
+      <c r="F90" s="40"/>
+      <c r="G90" s="40"/>
+      <c r="H90" s="40"/>
       <c r="I90" s="1"/>
       <c r="J90" s="39"/>
       <c r="K90" s="39"/>
@@ -4782,12 +4783,12 @@
       <c r="B94" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C94" s="43"/>
-      <c r="D94" s="43"/>
-      <c r="E94" s="43"/>
-      <c r="F94" s="43"/>
-      <c r="G94" s="43"/>
-      <c r="H94" s="43"/>
+      <c r="C94" s="40"/>
+      <c r="D94" s="40"/>
+      <c r="E94" s="40"/>
+      <c r="F94" s="40"/>
+      <c r="G94" s="40"/>
+      <c r="H94" s="40"/>
       <c r="I94" s="1"/>
       <c r="J94" s="39"/>
       <c r="K94" s="39"/>
@@ -4902,12 +4903,12 @@
       <c r="B98" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C98" s="43"/>
-      <c r="D98" s="43"/>
-      <c r="E98" s="43"/>
-      <c r="F98" s="43"/>
-      <c r="G98" s="43"/>
-      <c r="H98" s="43"/>
+      <c r="C98" s="40"/>
+      <c r="D98" s="40"/>
+      <c r="E98" s="40"/>
+      <c r="F98" s="40"/>
+      <c r="G98" s="40"/>
+      <c r="H98" s="40"/>
       <c r="I98" s="1"/>
       <c r="J98" s="39"/>
       <c r="K98" s="39"/>
@@ -5022,12 +5023,12 @@
       <c r="B102" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C102" s="43"/>
-      <c r="D102" s="43"/>
-      <c r="E102" s="43"/>
-      <c r="F102" s="43"/>
-      <c r="G102" s="43"/>
-      <c r="H102" s="43"/>
+      <c r="C102" s="40"/>
+      <c r="D102" s="40"/>
+      <c r="E102" s="40"/>
+      <c r="F102" s="40"/>
+      <c r="G102" s="40"/>
+      <c r="H102" s="40"/>
       <c r="I102" s="1"/>
       <c r="J102" s="39"/>
       <c r="K102" s="39"/>
@@ -5068,7 +5069,7 @@
       <c r="N103" s="1">
         <v>3.3446840501390498</v>
       </c>
-      <c r="O103" s="2">
+      <c r="O103" s="3">
         <v>7.0143959578357298E-2</v>
       </c>
       <c r="P103" s="1"/>
@@ -5406,12 +5407,12 @@
       <c r="B114" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C114" s="43"/>
-      <c r="D114" s="43"/>
-      <c r="E114" s="43"/>
-      <c r="F114" s="43"/>
-      <c r="G114" s="43"/>
-      <c r="H114" s="43"/>
+      <c r="C114" s="40"/>
+      <c r="D114" s="40"/>
+      <c r="E114" s="40"/>
+      <c r="F114" s="40"/>
+      <c r="G114" s="40"/>
+      <c r="H114" s="40"/>
       <c r="I114" s="1"/>
       <c r="J114" s="39"/>
       <c r="K114" s="39"/>
@@ -5526,12 +5527,12 @@
       <c r="B118" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C118" s="43"/>
-      <c r="D118" s="43"/>
-      <c r="E118" s="43"/>
-      <c r="F118" s="43"/>
-      <c r="G118" s="43"/>
-      <c r="H118" s="43"/>
+      <c r="C118" s="40"/>
+      <c r="D118" s="40"/>
+      <c r="E118" s="40"/>
+      <c r="F118" s="40"/>
+      <c r="G118" s="40"/>
+      <c r="H118" s="40"/>
       <c r="I118" s="1"/>
       <c r="J118" s="39"/>
       <c r="K118" s="39"/>
@@ -5646,12 +5647,12 @@
       <c r="B122" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C122" s="43"/>
-      <c r="D122" s="43"/>
-      <c r="E122" s="43"/>
-      <c r="F122" s="43"/>
-      <c r="G122" s="43"/>
-      <c r="H122" s="43"/>
+      <c r="C122" s="40"/>
+      <c r="D122" s="40"/>
+      <c r="E122" s="40"/>
+      <c r="F122" s="40"/>
+      <c r="G122" s="40"/>
+      <c r="H122" s="40"/>
       <c r="I122" s="1"/>
       <c r="J122" s="39"/>
       <c r="K122" s="39"/>
@@ -5766,12 +5767,12 @@
       <c r="B126" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C126" s="43"/>
-      <c r="D126" s="43"/>
-      <c r="E126" s="43"/>
-      <c r="F126" s="43"/>
-      <c r="G126" s="43"/>
-      <c r="H126" s="43"/>
+      <c r="C126" s="40"/>
+      <c r="D126" s="40"/>
+      <c r="E126" s="40"/>
+      <c r="F126" s="40"/>
+      <c r="G126" s="40"/>
+      <c r="H126" s="40"/>
       <c r="I126" s="1"/>
       <c r="J126" s="39"/>
       <c r="K126" s="39"/>
@@ -5886,12 +5887,12 @@
       <c r="B130" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C130" s="43"/>
-      <c r="D130" s="43"/>
-      <c r="E130" s="43"/>
-      <c r="F130" s="43"/>
-      <c r="G130" s="43"/>
-      <c r="H130" s="43"/>
+      <c r="C130" s="40"/>
+      <c r="D130" s="40"/>
+      <c r="E130" s="40"/>
+      <c r="F130" s="40"/>
+      <c r="G130" s="40"/>
+      <c r="H130" s="40"/>
       <c r="I130" s="1"/>
       <c r="J130" s="39"/>
       <c r="K130" s="39"/>
@@ -6006,12 +6007,12 @@
       <c r="B134" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C134" s="43"/>
-      <c r="D134" s="43"/>
-      <c r="E134" s="43"/>
-      <c r="F134" s="43"/>
-      <c r="G134" s="43"/>
-      <c r="H134" s="43"/>
+      <c r="C134" s="40"/>
+      <c r="D134" s="40"/>
+      <c r="E134" s="40"/>
+      <c r="F134" s="40"/>
+      <c r="G134" s="40"/>
+      <c r="H134" s="40"/>
       <c r="I134" s="1"/>
       <c r="J134" s="39"/>
       <c r="K134" s="39"/>
@@ -6126,12 +6127,12 @@
       <c r="B138" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C138" s="43"/>
-      <c r="D138" s="43"/>
-      <c r="E138" s="43"/>
-      <c r="F138" s="43"/>
-      <c r="G138" s="43"/>
-      <c r="H138" s="43"/>
+      <c r="C138" s="40"/>
+      <c r="D138" s="40"/>
+      <c r="E138" s="40"/>
+      <c r="F138" s="40"/>
+      <c r="G138" s="40"/>
+      <c r="H138" s="40"/>
       <c r="I138" s="1"/>
       <c r="J138" s="39"/>
       <c r="K138" s="39"/>
@@ -6161,68 +6162,14 @@
     </row>
   </sheetData>
   <mergeCells count="86">
-    <mergeCell ref="A15:A18"/>
-    <mergeCell ref="J15:O18"/>
-    <mergeCell ref="C18:H18"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C26:H26"/>
-    <mergeCell ref="C114:H114"/>
-    <mergeCell ref="C50:H50"/>
-    <mergeCell ref="C58:H58"/>
-    <mergeCell ref="C62:H62"/>
-    <mergeCell ref="C74:H74"/>
-    <mergeCell ref="C82:H82"/>
-    <mergeCell ref="C51:H54"/>
-    <mergeCell ref="J91:O94"/>
-    <mergeCell ref="J95:O98"/>
-    <mergeCell ref="J99:O102"/>
-    <mergeCell ref="C103:H106"/>
-    <mergeCell ref="C107:H110"/>
-    <mergeCell ref="C94:H94"/>
-    <mergeCell ref="C98:H98"/>
-    <mergeCell ref="C102:H102"/>
-    <mergeCell ref="J71:O74"/>
-    <mergeCell ref="C75:H78"/>
-    <mergeCell ref="J79:O82"/>
-    <mergeCell ref="C83:H86"/>
-    <mergeCell ref="J87:O90"/>
-    <mergeCell ref="C90:H90"/>
-    <mergeCell ref="J59:O62"/>
-    <mergeCell ref="C63:H66"/>
-    <mergeCell ref="C67:H70"/>
-    <mergeCell ref="C30:H30"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="C38:H38"/>
-    <mergeCell ref="C42:H42"/>
-    <mergeCell ref="C46:H46"/>
-    <mergeCell ref="J115:O118"/>
-    <mergeCell ref="J119:O122"/>
-    <mergeCell ref="J123:O126"/>
-    <mergeCell ref="J127:O130"/>
-    <mergeCell ref="C138:H138"/>
-    <mergeCell ref="C118:H118"/>
-    <mergeCell ref="C122:H122"/>
-    <mergeCell ref="C126:H126"/>
-    <mergeCell ref="C130:H130"/>
-    <mergeCell ref="C134:H134"/>
-    <mergeCell ref="J131:O134"/>
-    <mergeCell ref="J135:O138"/>
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="J1:P1"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="A7:A10"/>
-    <mergeCell ref="A11:A14"/>
-    <mergeCell ref="J11:O14"/>
-    <mergeCell ref="C6:H6"/>
-    <mergeCell ref="C10:H10"/>
-    <mergeCell ref="C14:H14"/>
-    <mergeCell ref="A19:A22"/>
-    <mergeCell ref="A23:A26"/>
-    <mergeCell ref="A27:A30"/>
-    <mergeCell ref="A31:A34"/>
-    <mergeCell ref="A35:A38"/>
-    <mergeCell ref="A39:A42"/>
-    <mergeCell ref="A43:A46"/>
+    <mergeCell ref="A107:A110"/>
+    <mergeCell ref="A131:A134"/>
+    <mergeCell ref="A135:A138"/>
+    <mergeCell ref="A111:A114"/>
+    <mergeCell ref="A115:A118"/>
+    <mergeCell ref="A119:A122"/>
+    <mergeCell ref="A123:A126"/>
+    <mergeCell ref="A127:A130"/>
     <mergeCell ref="A47:A50"/>
     <mergeCell ref="J111:O114"/>
     <mergeCell ref="A51:A54"/>
@@ -6239,14 +6186,68 @@
     <mergeCell ref="A95:A98"/>
     <mergeCell ref="A99:A102"/>
     <mergeCell ref="A103:A106"/>
-    <mergeCell ref="A107:A110"/>
-    <mergeCell ref="A131:A134"/>
-    <mergeCell ref="A135:A138"/>
-    <mergeCell ref="A111:A114"/>
-    <mergeCell ref="A115:A118"/>
-    <mergeCell ref="A119:A122"/>
-    <mergeCell ref="A123:A126"/>
-    <mergeCell ref="A127:A130"/>
+    <mergeCell ref="A27:A30"/>
+    <mergeCell ref="A31:A34"/>
+    <mergeCell ref="A35:A38"/>
+    <mergeCell ref="A39:A42"/>
+    <mergeCell ref="A43:A46"/>
+    <mergeCell ref="C1:I1"/>
+    <mergeCell ref="J1:P1"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="A7:A10"/>
+    <mergeCell ref="A11:A14"/>
+    <mergeCell ref="J11:O14"/>
+    <mergeCell ref="C6:H6"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C14:H14"/>
+    <mergeCell ref="J115:O118"/>
+    <mergeCell ref="J119:O122"/>
+    <mergeCell ref="J123:O126"/>
+    <mergeCell ref="J127:O130"/>
+    <mergeCell ref="C138:H138"/>
+    <mergeCell ref="C118:H118"/>
+    <mergeCell ref="C122:H122"/>
+    <mergeCell ref="C126:H126"/>
+    <mergeCell ref="C130:H130"/>
+    <mergeCell ref="C134:H134"/>
+    <mergeCell ref="J131:O134"/>
+    <mergeCell ref="J135:O138"/>
+    <mergeCell ref="J59:O62"/>
+    <mergeCell ref="C63:H66"/>
+    <mergeCell ref="C67:H70"/>
+    <mergeCell ref="C30:H30"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="C38:H38"/>
+    <mergeCell ref="C42:H42"/>
+    <mergeCell ref="C46:H46"/>
+    <mergeCell ref="J71:O74"/>
+    <mergeCell ref="C75:H78"/>
+    <mergeCell ref="J79:O82"/>
+    <mergeCell ref="C83:H86"/>
+    <mergeCell ref="J87:O90"/>
+    <mergeCell ref="C90:H90"/>
+    <mergeCell ref="J91:O94"/>
+    <mergeCell ref="J95:O98"/>
+    <mergeCell ref="J99:O102"/>
+    <mergeCell ref="C103:H106"/>
+    <mergeCell ref="C107:H110"/>
+    <mergeCell ref="C94:H94"/>
+    <mergeCell ref="C98:H98"/>
+    <mergeCell ref="C102:H102"/>
+    <mergeCell ref="C114:H114"/>
+    <mergeCell ref="C50:H50"/>
+    <mergeCell ref="C58:H58"/>
+    <mergeCell ref="C62:H62"/>
+    <mergeCell ref="C74:H74"/>
+    <mergeCell ref="C82:H82"/>
+    <mergeCell ref="C51:H54"/>
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="J15:O18"/>
+    <mergeCell ref="C18:H18"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C26:H26"/>
+    <mergeCell ref="A19:A22"/>
+    <mergeCell ref="A23:A26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -7071,22 +7072,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="40">
+      <c r="C1" s="41">
         <v>2021</v>
       </c>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="40">
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="41">
         <v>2022</v>
       </c>
-      <c r="J1" s="41"/>
-      <c r="K1" s="41"/>
-      <c r="L1" s="41"/>
-      <c r="M1" s="41"/>
-      <c r="N1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="43"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -9404,21 +9405,12 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="I1:N1"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="A7:A10"/>
-    <mergeCell ref="I3:M6"/>
-    <mergeCell ref="C7:G10"/>
-    <mergeCell ref="A19:A22"/>
-    <mergeCell ref="A23:A26"/>
-    <mergeCell ref="A11:A14"/>
-    <mergeCell ref="A15:A18"/>
-    <mergeCell ref="C1:H1"/>
-    <mergeCell ref="A39:A42"/>
-    <mergeCell ref="C39:G42"/>
-    <mergeCell ref="A27:A30"/>
-    <mergeCell ref="A31:A34"/>
-    <mergeCell ref="A35:A38"/>
+    <mergeCell ref="A63:A66"/>
+    <mergeCell ref="I63:M66"/>
+    <mergeCell ref="A67:A70"/>
+    <mergeCell ref="I67:M70"/>
+    <mergeCell ref="A59:A62"/>
+    <mergeCell ref="I59:M62"/>
     <mergeCell ref="A51:A54"/>
     <mergeCell ref="I51:M54"/>
     <mergeCell ref="A55:A58"/>
@@ -9427,12 +9419,21 @@
     <mergeCell ref="C43:G46"/>
     <mergeCell ref="A47:A50"/>
     <mergeCell ref="I47:M50"/>
-    <mergeCell ref="A63:A66"/>
-    <mergeCell ref="I63:M66"/>
-    <mergeCell ref="A67:A70"/>
-    <mergeCell ref="I67:M70"/>
-    <mergeCell ref="A59:A62"/>
-    <mergeCell ref="I59:M62"/>
+    <mergeCell ref="A39:A42"/>
+    <mergeCell ref="C39:G42"/>
+    <mergeCell ref="A27:A30"/>
+    <mergeCell ref="A31:A34"/>
+    <mergeCell ref="A35:A38"/>
+    <mergeCell ref="A19:A22"/>
+    <mergeCell ref="A23:A26"/>
+    <mergeCell ref="A11:A14"/>
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="C1:H1"/>
+    <mergeCell ref="I1:N1"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="A7:A10"/>
+    <mergeCell ref="I3:M6"/>
+    <mergeCell ref="C7:G10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>

<commit_message>
update Fruit Count to Basia Counts
</commit_message>
<xml_diff>
--- a/data/ModelResults.xlsx
+++ b/data/ModelResults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://michiganstate-my.sharepoint.com/personal/buysseso_msu_edu/Documents/Arabidopsis/Swe_Italy/R_scripts/SW_IT_PopDiffPlasticity/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1279" documentId="13_ncr:1_{AD4A5BE6-D9C1-414A-81C8-3A9C273D7774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2390976E-4F24-4B7F-A5C6-375CD9B01615}"/>
+  <xr:revisionPtr revIDLastSave="1360" documentId="13_ncr:1_{AD4A5BE6-D9C1-414A-81C8-3A9C273D7774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{359C411E-E97C-4AF5-A0DA-89B201753963}"/>
   <bookViews>
-    <workbookView xWindow="16095" yWindow="0" windowWidth="12705" windowHeight="15600" firstSheet="2" activeTab="3" xr2:uid="{8A213037-8BA5-417B-A75A-3088B4717938}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{8A213037-8BA5-417B-A75A-3088B4717938}"/>
   </bookViews>
   <sheets>
     <sheet name="ModelResults" sheetId="1" r:id="rId1"/>
@@ -143,9 +143,6 @@
     <t>Lat Branches</t>
   </si>
   <si>
-    <t>Fruit Number - log</t>
-  </si>
-  <si>
     <t>Fitness</t>
   </si>
   <si>
@@ -522,13 +519,16 @@
   </si>
   <si>
     <t>dry repro G - log - harvest</t>
+  </si>
+  <si>
+    <t>Fruit Number - BL counts</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -570,6 +570,12 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF009999"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -946,7 +952,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1036,6 +1042,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1043,9 +1052,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1087,6 +1093,16 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1463,24 +1479,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="53">
+      <c r="C1" s="54">
         <v>2021</v>
       </c>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="53">
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="54">
         <v>2022</v>
       </c>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
-      <c r="M1" s="54"/>
-      <c r="N1" s="54"/>
-      <c r="O1" s="54"/>
-      <c r="P1" s="55"/>
+      <c r="K1" s="55"/>
+      <c r="L1" s="55"/>
+      <c r="M1" s="55"/>
+      <c r="N1" s="55"/>
+      <c r="O1" s="55"/>
+      <c r="P1" s="56"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -1494,7 +1510,7 @@
         <v>3</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>4</v>
@@ -1506,7 +1522,7 @@
         <v>6</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>2</v>
@@ -1515,7 +1531,7 @@
         <v>3</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>4</v>
@@ -1527,12 +1543,12 @@
         <v>6</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="49" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>9</v>
@@ -1575,7 +1591,7 @@
         <v>2.27699983576885E-5</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -1669,14 +1685,14 @@
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="51"/>
       <c r="B6" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C6" s="56"/>
-      <c r="D6" s="56"/>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56"/>
-      <c r="G6" s="56"/>
-      <c r="H6" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C6" s="53"/>
+      <c r="D6" s="53"/>
+      <c r="E6" s="53"/>
+      <c r="F6" s="53"/>
+      <c r="G6" s="53"/>
+      <c r="H6" s="53"/>
       <c r="I6" s="1"/>
       <c r="J6" s="1">
         <v>3.5658276954852297E-2</v>
@@ -1700,7 +1716,7 @@
     </row>
     <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="49" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>9</v>
@@ -1835,14 +1851,14 @@
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="51"/>
       <c r="B10" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C10" s="56"/>
-      <c r="D10" s="56"/>
-      <c r="E10" s="56"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="56"/>
-      <c r="H10" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C10" s="53"/>
+      <c r="D10" s="53"/>
+      <c r="E10" s="53"/>
+      <c r="F10" s="53"/>
+      <c r="G10" s="53"/>
+      <c r="H10" s="53"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1">
         <v>8.3492792785920695</v>
@@ -1891,7 +1907,7 @@
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K11" s="52"/>
       <c r="L11" s="52"/>
@@ -1967,14 +1983,14 @@
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="51"/>
       <c r="B14" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="56"/>
-      <c r="D14" s="56"/>
-      <c r="E14" s="56"/>
-      <c r="F14" s="56"/>
-      <c r="G14" s="56"/>
-      <c r="H14" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C14" s="53"/>
+      <c r="D14" s="53"/>
+      <c r="E14" s="53"/>
+      <c r="F14" s="53"/>
+      <c r="G14" s="53"/>
+      <c r="H14" s="53"/>
       <c r="I14" s="1"/>
       <c r="J14" s="52"/>
       <c r="K14" s="52"/>
@@ -1986,7 +2002,7 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="49" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>9</v>
@@ -2011,7 +2027,7 @@
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K15" s="52"/>
       <c r="L15" s="52"/>
@@ -2086,14 +2102,14 @@
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="51"/>
       <c r="B18" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C18" s="56"/>
-      <c r="D18" s="56"/>
-      <c r="E18" s="56"/>
-      <c r="F18" s="56"/>
-      <c r="G18" s="56"/>
-      <c r="H18" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C18" s="53"/>
+      <c r="D18" s="53"/>
+      <c r="E18" s="53"/>
+      <c r="F18" s="53"/>
+      <c r="G18" s="53"/>
+      <c r="H18" s="53"/>
       <c r="I18" s="1"/>
       <c r="J18" s="52"/>
       <c r="K18" s="52"/>
@@ -2240,14 +2256,14 @@
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="51"/>
       <c r="B22" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C22" s="56"/>
-      <c r="D22" s="56"/>
-      <c r="E22" s="56"/>
-      <c r="F22" s="56"/>
-      <c r="G22" s="56"/>
-      <c r="H22" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C22" s="53"/>
+      <c r="D22" s="53"/>
+      <c r="E22" s="53"/>
+      <c r="F22" s="53"/>
+      <c r="G22" s="53"/>
+      <c r="H22" s="53"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1">
         <v>5.2456643231190104E-3</v>
@@ -2271,7 +2287,7 @@
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="49" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>9</v>
@@ -2406,14 +2422,14 @@
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="51"/>
       <c r="B26" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C26" s="56"/>
-      <c r="D26" s="56"/>
-      <c r="E26" s="56"/>
-      <c r="F26" s="56"/>
-      <c r="G26" s="56"/>
-      <c r="H26" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C26" s="53"/>
+      <c r="D26" s="53"/>
+      <c r="E26" s="53"/>
+      <c r="F26" s="53"/>
+      <c r="G26" s="53"/>
+      <c r="H26" s="53"/>
       <c r="I26" s="1"/>
       <c r="J26" s="1">
         <v>7.5239018444935397E-3</v>
@@ -2572,14 +2588,14 @@
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="51"/>
       <c r="B30" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C30" s="56"/>
-      <c r="D30" s="56"/>
-      <c r="E30" s="56"/>
-      <c r="F30" s="56"/>
-      <c r="G30" s="56"/>
-      <c r="H30" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C30" s="53"/>
+      <c r="D30" s="53"/>
+      <c r="E30" s="53"/>
+      <c r="F30" s="53"/>
+      <c r="G30" s="53"/>
+      <c r="H30" s="53"/>
       <c r="I30" s="1"/>
       <c r="J30" s="5">
         <v>7.2143853443936604E-6</v>
@@ -2738,14 +2754,14 @@
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" s="51"/>
       <c r="B34" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C34" s="56"/>
-      <c r="D34" s="56"/>
-      <c r="E34" s="56"/>
-      <c r="F34" s="56"/>
-      <c r="G34" s="56"/>
-      <c r="H34" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C34" s="53"/>
+      <c r="D34" s="53"/>
+      <c r="E34" s="53"/>
+      <c r="F34" s="53"/>
+      <c r="G34" s="53"/>
+      <c r="H34" s="53"/>
       <c r="I34" s="1"/>
       <c r="J34" s="1">
         <v>0.34951867520347901</v>
@@ -2904,14 +2920,14 @@
     <row r="38" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="51"/>
       <c r="B38" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C38" s="56"/>
-      <c r="D38" s="56"/>
-      <c r="E38" s="56"/>
-      <c r="F38" s="56"/>
-      <c r="G38" s="56"/>
-      <c r="H38" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C38" s="53"/>
+      <c r="D38" s="53"/>
+      <c r="E38" s="53"/>
+      <c r="F38" s="53"/>
+      <c r="G38" s="53"/>
+      <c r="H38" s="53"/>
       <c r="I38" s="1"/>
       <c r="J38" s="1">
         <v>2.5021778012642701</v>
@@ -3070,14 +3086,14 @@
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" s="51"/>
       <c r="B42" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C42" s="56"/>
-      <c r="D42" s="56"/>
-      <c r="E42" s="56"/>
-      <c r="F42" s="56"/>
-      <c r="G42" s="56"/>
-      <c r="H42" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C42" s="53"/>
+      <c r="D42" s="53"/>
+      <c r="E42" s="53"/>
+      <c r="F42" s="53"/>
+      <c r="G42" s="53"/>
+      <c r="H42" s="53"/>
       <c r="I42" s="1"/>
       <c r="J42" s="1">
         <v>4.9184876384352101E-2</v>
@@ -3236,14 +3252,14 @@
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="51"/>
       <c r="B46" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C46" s="56"/>
-      <c r="D46" s="56"/>
-      <c r="E46" s="56"/>
-      <c r="F46" s="56"/>
-      <c r="G46" s="56"/>
-      <c r="H46" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C46" s="53"/>
+      <c r="D46" s="53"/>
+      <c r="E46" s="53"/>
+      <c r="F46" s="53"/>
+      <c r="G46" s="53"/>
+      <c r="H46" s="53"/>
       <c r="I46" s="1"/>
       <c r="J46" s="1">
         <v>3.6858467316493698E-2</v>
@@ -3402,14 +3418,14 @@
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="51"/>
       <c r="B50" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C50" s="56"/>
-      <c r="D50" s="56"/>
-      <c r="E50" s="56"/>
-      <c r="F50" s="56"/>
-      <c r="G50" s="56"/>
-      <c r="H50" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C50" s="53"/>
+      <c r="D50" s="53"/>
+      <c r="E50" s="53"/>
+      <c r="F50" s="53"/>
+      <c r="G50" s="53"/>
+      <c r="H50" s="53"/>
       <c r="I50" s="1"/>
       <c r="J50" s="1">
         <v>3.4846897009296399E-3</v>
@@ -3433,13 +3449,13 @@
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="49" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C51" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D51" s="52"/>
       <c r="E51" s="52"/>
@@ -3534,7 +3550,7 @@
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="51"/>
       <c r="B54" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C54" s="52"/>
       <c r="D54" s="52"/>
@@ -3565,7 +3581,7 @@
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" s="49" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>9</v>
@@ -3608,7 +3624,7 @@
         <v>5.4997814524115098E-3</v>
       </c>
       <c r="P55" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
@@ -3702,14 +3718,14 @@
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" s="51"/>
       <c r="B58" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C58" s="56"/>
-      <c r="D58" s="56"/>
-      <c r="E58" s="56"/>
-      <c r="F58" s="56"/>
-      <c r="G58" s="56"/>
-      <c r="H58" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C58" s="53"/>
+      <c r="D58" s="53"/>
+      <c r="E58" s="53"/>
+      <c r="F58" s="53"/>
+      <c r="G58" s="53"/>
+      <c r="H58" s="53"/>
       <c r="I58" s="1"/>
       <c r="J58" s="1">
         <v>1.0524858270047699</v>
@@ -3733,7 +3749,7 @@
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" s="49" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>9</v>
@@ -3758,7 +3774,7 @@
       </c>
       <c r="I59" s="1"/>
       <c r="J59" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K59" s="52"/>
       <c r="L59" s="52"/>
@@ -3834,14 +3850,14 @@
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" s="51"/>
       <c r="B62" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C62" s="56"/>
-      <c r="D62" s="56"/>
-      <c r="E62" s="56"/>
-      <c r="F62" s="56"/>
-      <c r="G62" s="56"/>
-      <c r="H62" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C62" s="53"/>
+      <c r="D62" s="53"/>
+      <c r="E62" s="53"/>
+      <c r="F62" s="53"/>
+      <c r="G62" s="53"/>
+      <c r="H62" s="53"/>
       <c r="I62" s="1"/>
       <c r="J62" s="52"/>
       <c r="K62" s="52"/>
@@ -3853,13 +3869,13 @@
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" s="49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B63" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C63" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D63" s="52"/>
       <c r="E63" s="52"/>
@@ -3954,7 +3970,7 @@
     <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" s="51"/>
       <c r="B66" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C66" s="52"/>
       <c r="D66" s="52"/>
@@ -3985,13 +4001,13 @@
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="49" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B67" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C67" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D67" s="52"/>
       <c r="E67" s="52"/>
@@ -4086,7 +4102,7 @@
     <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="51"/>
       <c r="B70" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C70" s="52"/>
       <c r="D70" s="52"/>
@@ -4117,7 +4133,7 @@
     </row>
     <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" s="49" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>9</v>
@@ -4142,7 +4158,7 @@
       </c>
       <c r="I71" s="1"/>
       <c r="J71" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K71" s="52"/>
       <c r="L71" s="52"/>
@@ -4218,14 +4234,14 @@
     <row r="74" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="51"/>
       <c r="B74" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C74" s="56"/>
-      <c r="D74" s="56"/>
-      <c r="E74" s="56"/>
-      <c r="F74" s="56"/>
-      <c r="G74" s="56"/>
-      <c r="H74" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C74" s="53"/>
+      <c r="D74" s="53"/>
+      <c r="E74" s="53"/>
+      <c r="F74" s="53"/>
+      <c r="G74" s="53"/>
+      <c r="H74" s="53"/>
       <c r="I74" s="1"/>
       <c r="J74" s="52"/>
       <c r="K74" s="52"/>
@@ -4243,7 +4259,7 @@
         <v>9</v>
       </c>
       <c r="C75" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D75" s="52"/>
       <c r="E75" s="52"/>
@@ -4338,7 +4354,7 @@
     <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" s="51"/>
       <c r="B78" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C78" s="52"/>
       <c r="D78" s="52"/>
@@ -4394,7 +4410,7 @@
       </c>
       <c r="I79" s="1"/>
       <c r="J79" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K79" s="52"/>
       <c r="L79" s="52"/>
@@ -4470,14 +4486,14 @@
     <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82" s="51"/>
       <c r="B82" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C82" s="56"/>
-      <c r="D82" s="56"/>
-      <c r="E82" s="56"/>
-      <c r="F82" s="56"/>
-      <c r="G82" s="56"/>
-      <c r="H82" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C82" s="53"/>
+      <c r="D82" s="53"/>
+      <c r="E82" s="53"/>
+      <c r="F82" s="53"/>
+      <c r="G82" s="53"/>
+      <c r="H82" s="53"/>
       <c r="I82" s="1"/>
       <c r="J82" s="52"/>
       <c r="K82" s="52"/>
@@ -4489,13 +4505,13 @@
     </row>
     <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83" s="49" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B83" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C83" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D83" s="52"/>
       <c r="E83" s="52"/>
@@ -4590,7 +4606,7 @@
     <row r="86" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A86" s="51"/>
       <c r="B86" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C86" s="52"/>
       <c r="D86" s="52"/>
@@ -4621,7 +4637,7 @@
     </row>
     <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87" s="49" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B87" s="1" t="s">
         <v>9</v>
@@ -4646,7 +4662,7 @@
       </c>
       <c r="I87" s="1"/>
       <c r="J87" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K87" s="52"/>
       <c r="L87" s="52"/>
@@ -4722,14 +4738,14 @@
     <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A90" s="51"/>
       <c r="B90" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C90" s="56"/>
-      <c r="D90" s="56"/>
-      <c r="E90" s="56"/>
-      <c r="F90" s="56"/>
-      <c r="G90" s="56"/>
-      <c r="H90" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C90" s="53"/>
+      <c r="D90" s="53"/>
+      <c r="E90" s="53"/>
+      <c r="F90" s="53"/>
+      <c r="G90" s="53"/>
+      <c r="H90" s="53"/>
       <c r="I90" s="1"/>
       <c r="J90" s="52"/>
       <c r="K90" s="52"/>
@@ -4766,7 +4782,7 @@
       </c>
       <c r="I91" s="1"/>
       <c r="J91" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K91" s="52"/>
       <c r="L91" s="52"/>
@@ -4842,14 +4858,14 @@
     <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A94" s="51"/>
       <c r="B94" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C94" s="56"/>
-      <c r="D94" s="56"/>
-      <c r="E94" s="56"/>
-      <c r="F94" s="56"/>
-      <c r="G94" s="56"/>
-      <c r="H94" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C94" s="53"/>
+      <c r="D94" s="53"/>
+      <c r="E94" s="53"/>
+      <c r="F94" s="53"/>
+      <c r="G94" s="53"/>
+      <c r="H94" s="53"/>
       <c r="I94" s="1"/>
       <c r="J94" s="52"/>
       <c r="K94" s="52"/>
@@ -4886,7 +4902,7 @@
       </c>
       <c r="I95" s="1"/>
       <c r="J95" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K95" s="52"/>
       <c r="L95" s="52"/>
@@ -4962,14 +4978,14 @@
     <row r="98" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A98" s="51"/>
       <c r="B98" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C98" s="56"/>
-      <c r="D98" s="56"/>
-      <c r="E98" s="56"/>
-      <c r="F98" s="56"/>
-      <c r="G98" s="56"/>
-      <c r="H98" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C98" s="53"/>
+      <c r="D98" s="53"/>
+      <c r="E98" s="53"/>
+      <c r="F98" s="53"/>
+      <c r="G98" s="53"/>
+      <c r="H98" s="53"/>
       <c r="I98" s="1"/>
       <c r="J98" s="52"/>
       <c r="K98" s="52"/>
@@ -4981,7 +4997,7 @@
     </row>
     <row r="99" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A99" s="49" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B99" s="1" t="s">
         <v>9</v>
@@ -5006,7 +5022,7 @@
       </c>
       <c r="I99" s="1"/>
       <c r="J99" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K99" s="52"/>
       <c r="L99" s="52"/>
@@ -5082,14 +5098,14 @@
     <row r="102" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A102" s="51"/>
       <c r="B102" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C102" s="56"/>
-      <c r="D102" s="56"/>
-      <c r="E102" s="56"/>
-      <c r="F102" s="56"/>
-      <c r="G102" s="56"/>
-      <c r="H102" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C102" s="53"/>
+      <c r="D102" s="53"/>
+      <c r="E102" s="53"/>
+      <c r="F102" s="53"/>
+      <c r="G102" s="53"/>
+      <c r="H102" s="53"/>
       <c r="I102" s="1"/>
       <c r="J102" s="52"/>
       <c r="K102" s="52"/>
@@ -5101,13 +5117,13 @@
     </row>
     <row r="103" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A103" s="49" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B103" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C103" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D103" s="52"/>
       <c r="E103" s="52"/>
@@ -5202,7 +5218,7 @@
     <row r="106" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A106" s="51"/>
       <c r="B106" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C106" s="52"/>
       <c r="D106" s="52"/>
@@ -5233,13 +5249,13 @@
     </row>
     <row r="107" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A107" s="49" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B107" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C107" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D107" s="52"/>
       <c r="E107" s="52"/>
@@ -5334,7 +5350,7 @@
     <row r="110" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A110" s="51"/>
       <c r="B110" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C110" s="52"/>
       <c r="D110" s="52"/>
@@ -5390,7 +5406,7 @@
       </c>
       <c r="I111" s="1"/>
       <c r="J111" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K111" s="52"/>
       <c r="L111" s="52"/>
@@ -5466,14 +5482,14 @@
     <row r="114" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A114" s="51"/>
       <c r="B114" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C114" s="56"/>
-      <c r="D114" s="56"/>
-      <c r="E114" s="56"/>
-      <c r="F114" s="56"/>
-      <c r="G114" s="56"/>
-      <c r="H114" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C114" s="53"/>
+      <c r="D114" s="53"/>
+      <c r="E114" s="53"/>
+      <c r="F114" s="53"/>
+      <c r="G114" s="53"/>
+      <c r="H114" s="53"/>
       <c r="I114" s="1"/>
       <c r="J114" s="52"/>
       <c r="K114" s="52"/>
@@ -5510,7 +5526,7 @@
       </c>
       <c r="I115" s="1"/>
       <c r="J115" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K115" s="52"/>
       <c r="L115" s="52"/>
@@ -5586,14 +5602,14 @@
     <row r="118" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A118" s="51"/>
       <c r="B118" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C118" s="56"/>
-      <c r="D118" s="56"/>
-      <c r="E118" s="56"/>
-      <c r="F118" s="56"/>
-      <c r="G118" s="56"/>
-      <c r="H118" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C118" s="53"/>
+      <c r="D118" s="53"/>
+      <c r="E118" s="53"/>
+      <c r="F118" s="53"/>
+      <c r="G118" s="53"/>
+      <c r="H118" s="53"/>
       <c r="I118" s="1"/>
       <c r="J118" s="52"/>
       <c r="K118" s="52"/>
@@ -5630,7 +5646,7 @@
       </c>
       <c r="I119" s="1"/>
       <c r="J119" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K119" s="52"/>
       <c r="L119" s="52"/>
@@ -5706,14 +5722,14 @@
     <row r="122" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A122" s="51"/>
       <c r="B122" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C122" s="56"/>
-      <c r="D122" s="56"/>
-      <c r="E122" s="56"/>
-      <c r="F122" s="56"/>
-      <c r="G122" s="56"/>
-      <c r="H122" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C122" s="53"/>
+      <c r="D122" s="53"/>
+      <c r="E122" s="53"/>
+      <c r="F122" s="53"/>
+      <c r="G122" s="53"/>
+      <c r="H122" s="53"/>
       <c r="I122" s="1"/>
       <c r="J122" s="52"/>
       <c r="K122" s="52"/>
@@ -5724,33 +5740,33 @@
       <c r="P122" s="1"/>
     </row>
     <row r="123" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A123" s="49" t="s">
-        <v>25</v>
+      <c r="A123" s="70" t="s">
+        <v>151</v>
       </c>
       <c r="B123" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C123" s="1">
-        <v>8.1889606725674895</v>
+        <v>6176915.5049999999</v>
       </c>
       <c r="D123" s="1">
-        <v>8.1889606725674895</v>
+        <v>6176915.5049999999</v>
       </c>
       <c r="E123" s="1">
         <v>1</v>
       </c>
       <c r="F123" s="1">
-        <v>38.960439075121599</v>
+        <v>71.888440000000003</v>
       </c>
       <c r="G123" s="1">
-        <v>229.518131380033</v>
+        <v>167.3449876</v>
       </c>
       <c r="H123" s="4">
-        <v>6.3990332076812E-18</v>
+        <v>1.898803E-20</v>
       </c>
       <c r="I123" s="1"/>
       <c r="J123" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K123" s="52"/>
       <c r="L123" s="52"/>
@@ -5760,27 +5776,27 @@
       <c r="P123" s="1"/>
     </row>
     <row r="124" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A124" s="50"/>
+      <c r="A124" s="71"/>
       <c r="B124" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C124" s="1">
-        <v>0.23039707874839899</v>
+        <v>50157.928</v>
       </c>
       <c r="D124" s="1">
-        <v>0.23039707874839899</v>
+        <v>50157.928</v>
       </c>
       <c r="E124" s="1">
         <v>1</v>
       </c>
       <c r="F124" s="1">
-        <v>4.1944106114323096</v>
+        <v>17.04102</v>
       </c>
       <c r="G124" s="1">
-        <v>6.45751141129504</v>
-      </c>
-      <c r="H124" s="3">
-        <v>6.1070966449770503E-2</v>
+        <v>1.3588785000000001</v>
+      </c>
+      <c r="H124" s="1">
+        <v>0.2597892</v>
       </c>
       <c r="I124" s="1"/>
       <c r="J124" s="52"/>
@@ -5792,27 +5808,27 @@
       <c r="P124" s="1"/>
     </row>
     <row r="125" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A125" s="50"/>
+      <c r="A125" s="71"/>
       <c r="B125" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C125" s="1">
-        <v>0.24741116524293899</v>
+        <v>5310.1710000000003</v>
       </c>
       <c r="D125" s="1">
-        <v>0.24741116524293899</v>
+        <v>5310.1710000000003</v>
       </c>
       <c r="E125" s="1">
         <v>1</v>
       </c>
       <c r="F125" s="1">
-        <v>38.960439070902197</v>
+        <v>71.888440000000003</v>
       </c>
       <c r="G125" s="1">
-        <v>6.9343779509581998</v>
-      </c>
-      <c r="H125" s="2">
-        <v>1.2062369794193201E-2</v>
+        <v>0.1438632</v>
+      </c>
+      <c r="H125" s="1">
+        <v>0.7055884</v>
       </c>
       <c r="I125" s="1"/>
       <c r="J125" s="52"/>
@@ -5824,16 +5840,16 @@
       <c r="P125" s="1"/>
     </row>
     <row r="126" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A126" s="51"/>
+      <c r="A126" s="72"/>
       <c r="B126" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C126" s="56"/>
-      <c r="D126" s="56"/>
-      <c r="E126" s="56"/>
-      <c r="F126" s="56"/>
-      <c r="G126" s="56"/>
-      <c r="H126" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C126" s="53"/>
+      <c r="D126" s="53"/>
+      <c r="E126" s="53"/>
+      <c r="F126" s="53"/>
+      <c r="G126" s="53"/>
+      <c r="H126" s="53"/>
       <c r="I126" s="1"/>
       <c r="J126" s="52"/>
       <c r="K126" s="52"/>
@@ -5845,7 +5861,7 @@
     </row>
     <row r="127" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A127" s="49" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B127" s="1" t="s">
         <v>9</v>
@@ -5870,7 +5886,7 @@
       </c>
       <c r="I127" s="1"/>
       <c r="J127" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K127" s="52"/>
       <c r="L127" s="52"/>
@@ -5946,14 +5962,14 @@
     <row r="130" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A130" s="51"/>
       <c r="B130" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C130" s="56"/>
-      <c r="D130" s="56"/>
-      <c r="E130" s="56"/>
-      <c r="F130" s="56"/>
-      <c r="G130" s="56"/>
-      <c r="H130" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C130" s="53"/>
+      <c r="D130" s="53"/>
+      <c r="E130" s="53"/>
+      <c r="F130" s="53"/>
+      <c r="G130" s="53"/>
+      <c r="H130" s="53"/>
       <c r="I130" s="1"/>
       <c r="J130" s="52"/>
       <c r="K130" s="52"/>
@@ -5965,7 +5981,7 @@
     </row>
     <row r="131" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A131" s="49" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B131" s="1" t="s">
         <v>9</v>
@@ -5990,7 +6006,7 @@
       </c>
       <c r="I131" s="1"/>
       <c r="J131" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K131" s="52"/>
       <c r="L131" s="52"/>
@@ -6066,14 +6082,14 @@
     <row r="134" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A134" s="51"/>
       <c r="B134" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C134" s="56"/>
-      <c r="D134" s="56"/>
-      <c r="E134" s="56"/>
-      <c r="F134" s="56"/>
-      <c r="G134" s="56"/>
-      <c r="H134" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C134" s="53"/>
+      <c r="D134" s="53"/>
+      <c r="E134" s="53"/>
+      <c r="F134" s="53"/>
+      <c r="G134" s="53"/>
+      <c r="H134" s="53"/>
       <c r="I134" s="1"/>
       <c r="J134" s="52"/>
       <c r="K134" s="52"/>
@@ -6085,32 +6101,32 @@
     </row>
     <row r="135" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A135" s="49" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B135" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C135" s="1">
-        <v>11.0082179168385</v>
+        <v>11.200752100000001</v>
       </c>
       <c r="D135" s="1">
-        <v>11.0082179168385</v>
+        <v>11.200752100000001</v>
       </c>
       <c r="E135" s="1">
         <v>1</v>
       </c>
       <c r="F135" s="1">
-        <v>48.794824022977402</v>
+        <v>51.667794999999998</v>
       </c>
       <c r="G135" s="1">
-        <v>408.97170017139501</v>
+        <v>471.893664</v>
       </c>
       <c r="H135" s="4">
-        <v>2.2809234413835001E-25</v>
+        <v>1.209274E-27</v>
       </c>
       <c r="I135" s="1"/>
       <c r="J135" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K135" s="52"/>
       <c r="L135" s="52"/>
@@ -6125,22 +6141,22 @@
         <v>7</v>
       </c>
       <c r="C136" s="1">
-        <v>0.12480779741629899</v>
+        <v>0.12802530000000001</v>
       </c>
       <c r="D136" s="1">
-        <v>0.12480779741629899</v>
+        <v>0.12802530000000001</v>
       </c>
       <c r="E136" s="1">
         <v>1</v>
       </c>
       <c r="F136" s="1">
-        <v>6.2935571141001798</v>
+        <v>6.2246040000000002</v>
       </c>
       <c r="G136" s="1">
-        <v>4.6367956638934302</v>
-      </c>
-      <c r="H136" s="3">
-        <v>7.2640986050278702E-2</v>
+        <v>5.3937730000000004</v>
+      </c>
+      <c r="H136" s="4">
+        <v>5.7713939999999998E-2</v>
       </c>
       <c r="I136" s="1"/>
       <c r="J136" s="52"/>
@@ -6157,22 +6173,22 @@
         <v>8</v>
       </c>
       <c r="C137" s="1">
-        <v>0.74925429491560802</v>
+        <v>0.70815150000000004</v>
       </c>
       <c r="D137" s="1">
-        <v>0.74925429491560802</v>
+        <v>0.70815150000000004</v>
       </c>
       <c r="E137" s="1">
         <v>1</v>
       </c>
       <c r="F137" s="1">
-        <v>48.794824017520803</v>
+        <v>51.667794999999998</v>
       </c>
       <c r="G137" s="1">
-        <v>27.8359136026586</v>
+        <v>29.834802</v>
       </c>
       <c r="H137" s="4">
-        <v>3.01236497113781E-6</v>
+        <v>1.363103E-6</v>
       </c>
       <c r="I137" s="1"/>
       <c r="J137" s="52"/>
@@ -6186,14 +6202,14 @@
     <row r="138" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A138" s="51"/>
       <c r="B138" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C138" s="56"/>
-      <c r="D138" s="56"/>
-      <c r="E138" s="56"/>
-      <c r="F138" s="56"/>
-      <c r="G138" s="56"/>
-      <c r="H138" s="56"/>
+        <v>37</v>
+      </c>
+      <c r="C138" s="53"/>
+      <c r="D138" s="53"/>
+      <c r="E138" s="53"/>
+      <c r="F138" s="53"/>
+      <c r="G138" s="53"/>
+      <c r="H138" s="53"/>
       <c r="I138" s="1"/>
       <c r="J138" s="52"/>
       <c r="K138" s="52"/>
@@ -6223,68 +6239,14 @@
     </row>
   </sheetData>
   <mergeCells count="86">
-    <mergeCell ref="A15:A18"/>
-    <mergeCell ref="J15:O18"/>
-    <mergeCell ref="C18:H18"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C26:H26"/>
-    <mergeCell ref="A19:A22"/>
-    <mergeCell ref="A23:A26"/>
-    <mergeCell ref="C114:H114"/>
-    <mergeCell ref="C50:H50"/>
-    <mergeCell ref="C58:H58"/>
-    <mergeCell ref="C62:H62"/>
-    <mergeCell ref="C74:H74"/>
-    <mergeCell ref="C82:H82"/>
-    <mergeCell ref="C51:H54"/>
-    <mergeCell ref="J91:O94"/>
-    <mergeCell ref="J95:O98"/>
-    <mergeCell ref="J99:O102"/>
-    <mergeCell ref="C103:H106"/>
-    <mergeCell ref="C107:H110"/>
-    <mergeCell ref="C94:H94"/>
-    <mergeCell ref="C98:H98"/>
-    <mergeCell ref="C102:H102"/>
-    <mergeCell ref="J71:O74"/>
-    <mergeCell ref="C75:H78"/>
-    <mergeCell ref="J79:O82"/>
-    <mergeCell ref="C83:H86"/>
-    <mergeCell ref="J87:O90"/>
-    <mergeCell ref="C90:H90"/>
-    <mergeCell ref="J59:O62"/>
-    <mergeCell ref="C63:H66"/>
-    <mergeCell ref="C67:H70"/>
-    <mergeCell ref="C30:H30"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="C38:H38"/>
-    <mergeCell ref="C42:H42"/>
-    <mergeCell ref="C46:H46"/>
-    <mergeCell ref="J115:O118"/>
-    <mergeCell ref="J119:O122"/>
-    <mergeCell ref="J123:O126"/>
-    <mergeCell ref="J127:O130"/>
-    <mergeCell ref="C138:H138"/>
-    <mergeCell ref="C118:H118"/>
-    <mergeCell ref="C122:H122"/>
-    <mergeCell ref="C126:H126"/>
-    <mergeCell ref="C130:H130"/>
-    <mergeCell ref="C134:H134"/>
-    <mergeCell ref="J131:O134"/>
-    <mergeCell ref="J135:O138"/>
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="J1:P1"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="A7:A10"/>
-    <mergeCell ref="A11:A14"/>
-    <mergeCell ref="J11:O14"/>
-    <mergeCell ref="C6:H6"/>
-    <mergeCell ref="C10:H10"/>
-    <mergeCell ref="C14:H14"/>
-    <mergeCell ref="A27:A30"/>
-    <mergeCell ref="A31:A34"/>
-    <mergeCell ref="A35:A38"/>
-    <mergeCell ref="A39:A42"/>
-    <mergeCell ref="A43:A46"/>
+    <mergeCell ref="A107:A110"/>
+    <mergeCell ref="A131:A134"/>
+    <mergeCell ref="A135:A138"/>
+    <mergeCell ref="A111:A114"/>
+    <mergeCell ref="A115:A118"/>
+    <mergeCell ref="A119:A122"/>
+    <mergeCell ref="A123:A126"/>
+    <mergeCell ref="A127:A130"/>
     <mergeCell ref="A47:A50"/>
     <mergeCell ref="J111:O114"/>
     <mergeCell ref="A51:A54"/>
@@ -6301,14 +6263,68 @@
     <mergeCell ref="A95:A98"/>
     <mergeCell ref="A99:A102"/>
     <mergeCell ref="A103:A106"/>
-    <mergeCell ref="A107:A110"/>
-    <mergeCell ref="A131:A134"/>
-    <mergeCell ref="A135:A138"/>
-    <mergeCell ref="A111:A114"/>
-    <mergeCell ref="A115:A118"/>
-    <mergeCell ref="A119:A122"/>
-    <mergeCell ref="A123:A126"/>
-    <mergeCell ref="A127:A130"/>
+    <mergeCell ref="A27:A30"/>
+    <mergeCell ref="A31:A34"/>
+    <mergeCell ref="A35:A38"/>
+    <mergeCell ref="A39:A42"/>
+    <mergeCell ref="A43:A46"/>
+    <mergeCell ref="C1:I1"/>
+    <mergeCell ref="J1:P1"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="A7:A10"/>
+    <mergeCell ref="A11:A14"/>
+    <mergeCell ref="J11:O14"/>
+    <mergeCell ref="C6:H6"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C14:H14"/>
+    <mergeCell ref="J115:O118"/>
+    <mergeCell ref="J119:O122"/>
+    <mergeCell ref="J123:O126"/>
+    <mergeCell ref="J127:O130"/>
+    <mergeCell ref="C138:H138"/>
+    <mergeCell ref="C118:H118"/>
+    <mergeCell ref="C122:H122"/>
+    <mergeCell ref="C126:H126"/>
+    <mergeCell ref="C130:H130"/>
+    <mergeCell ref="C134:H134"/>
+    <mergeCell ref="J131:O134"/>
+    <mergeCell ref="J135:O138"/>
+    <mergeCell ref="J59:O62"/>
+    <mergeCell ref="C63:H66"/>
+    <mergeCell ref="C67:H70"/>
+    <mergeCell ref="C30:H30"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="C38:H38"/>
+    <mergeCell ref="C42:H42"/>
+    <mergeCell ref="C46:H46"/>
+    <mergeCell ref="J71:O74"/>
+    <mergeCell ref="C75:H78"/>
+    <mergeCell ref="J79:O82"/>
+    <mergeCell ref="C83:H86"/>
+    <mergeCell ref="J87:O90"/>
+    <mergeCell ref="C90:H90"/>
+    <mergeCell ref="J91:O94"/>
+    <mergeCell ref="J95:O98"/>
+    <mergeCell ref="J99:O102"/>
+    <mergeCell ref="C103:H106"/>
+    <mergeCell ref="C107:H110"/>
+    <mergeCell ref="C94:H94"/>
+    <mergeCell ref="C98:H98"/>
+    <mergeCell ref="C102:H102"/>
+    <mergeCell ref="C114:H114"/>
+    <mergeCell ref="C50:H50"/>
+    <mergeCell ref="C58:H58"/>
+    <mergeCell ref="C62:H62"/>
+    <mergeCell ref="C74:H74"/>
+    <mergeCell ref="C82:H82"/>
+    <mergeCell ref="C51:H54"/>
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="J15:O18"/>
+    <mergeCell ref="C18:H18"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C26:H26"/>
+    <mergeCell ref="A19:A22"/>
+    <mergeCell ref="A23:A26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6336,28 +6352,28 @@
     <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="12"/>
       <c r="B1" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="D1" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="E1" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="E1" s="12" t="s">
-        <v>47</v>
-      </c>
       <c r="F1" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I1" s="12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L1" s="6"/>
     </row>
@@ -6367,21 +6383,20 @@
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E2" s="13"/>
       <c r="F2" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="G2" s="13"/>
+        <v>50</v>
+      </c>
       <c r="H2" s="28" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I2" s="29" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L2" s="6"/>
     </row>
@@ -6390,18 +6405,18 @@
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -6409,18 +6424,18 @@
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I4" s="30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L4" s="6"/>
     </row>
@@ -6429,18 +6444,18 @@
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="24" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I5" s="27" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L5" s="6"/>
     </row>
@@ -6448,17 +6463,19 @@
       <c r="A6" s="58"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
+      <c r="D6" s="73" t="s">
+        <v>74</v>
+      </c>
       <c r="E6" s="1"/>
       <c r="F6" s="20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="32" t="s">
         <v>17</v>
       </c>
       <c r="I6" s="33" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -6468,14 +6485,11 @@
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="I7" s="26" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="L7" s="6"/>
     </row>
@@ -6486,12 +6500,12 @@
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="27" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L8" s="6"/>
     </row>
@@ -6501,17 +6515,16 @@
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="33" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J9" s="24" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6525,7 +6538,7 @@
       <c r="H10" s="16"/>
       <c r="I10" s="17"/>
       <c r="J10" s="25" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -6534,47 +6547,47 @@
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E11" s="13"/>
       <c r="F11" s="22" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G11" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="H11" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="I11" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="H11" s="34" t="s">
-        <v>57</v>
-      </c>
-      <c r="I11" s="23" t="s">
-        <v>88</v>
-      </c>
       <c r="J11" s="18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="58"/>
       <c r="B12" s="1"/>
       <c r="C12" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>82</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I12" s="27" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
@@ -6582,16 +6595,16 @@
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="27" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -6604,7 +6617,7 @@
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
       <c r="I14" s="21" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -6617,7 +6630,7 @@
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="31" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -6630,7 +6643,7 @@
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="30" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6656,7 @@
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="26" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6659,70 +6672,70 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>98</v>
+      </c>
+      <c r="B29" t="s">
         <v>99</v>
-      </c>
-      <c r="B29" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -6753,28 +6766,28 @@
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="12"/>
       <c r="B1" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="D1" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="D1" s="12" t="s">
-        <v>46</v>
-      </c>
       <c r="E1" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I1" s="35" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K1" s="6"/>
     </row>
@@ -6784,20 +6797,20 @@
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F2" s="13"/>
       <c r="G2" s="32" t="s">
         <v>17</v>
       </c>
       <c r="H2" s="30" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K2" s="6"/>
     </row>
@@ -6805,14 +6818,16 @@
       <c r="A3" s="58"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
+      <c r="D3" s="73" t="s">
+        <v>74</v>
+      </c>
       <c r="E3" s="20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="24"/>
       <c r="H3" s="30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -6820,12 +6835,12 @@
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="E4" s="20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="24"/>
       <c r="H4" s="27" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="K4" s="6"/>
     </row>
@@ -6835,13 +6850,10 @@
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="24"/>
-      <c r="H5" s="26" t="s">
-        <v>75</v>
-      </c>
       <c r="K5" s="6"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -6850,11 +6862,11 @@
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F6" s="1"/>
       <c r="H6" s="27" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -6862,11 +6874,10 @@
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="32"/>
       <c r="H7" s="33" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K7" s="6"/>
     </row>
@@ -6891,10 +6902,10 @@
       <c r="G9" s="1"/>
       <c r="H9" s="26"/>
       <c r="I9" s="24" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6907,7 +6918,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="17"/>
       <c r="I10" s="25" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -6918,31 +6929,31 @@
       <c r="C11" s="13"/>
       <c r="D11" s="19"/>
       <c r="E11" s="19" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G11" s="34"/>
       <c r="H11" s="23"/>
       <c r="I11" s="18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="58"/>
       <c r="B12" s="1"/>
       <c r="C12" s="20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="25"/>
       <c r="H12" s="31" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -6953,7 +6964,7 @@
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
       <c r="H13" s="31" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -6965,7 +6976,7 @@
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="30" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -6977,7 +6988,7 @@
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="26" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -7012,87 +7023,87 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="37" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -7133,24 +7144,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="C1" s="53">
+        <v>142</v>
+      </c>
+      <c r="C1" s="54">
         <v>2021</v>
       </c>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="53">
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="54">
         <v>2022</v>
       </c>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
-      <c r="M1" s="54"/>
-      <c r="N1" s="55"/>
+      <c r="J1" s="55"/>
+      <c r="K1" s="55"/>
+      <c r="L1" s="55"/>
+      <c r="M1" s="55"/>
+      <c r="N1" s="56"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -7158,48 +7169,48 @@
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>115</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>115</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="49" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C3" s="1">
         <v>3.5206400000000002</v>
@@ -7218,7 +7229,7 @@
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="61" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J3" s="62"/>
       <c r="K3" s="62"/>
@@ -7229,7 +7240,7 @@
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="50"/>
       <c r="B4" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C4" s="1">
         <v>1.189046</v>
@@ -7257,7 +7268,7 @@
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="50"/>
       <c r="B5" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C5" s="1">
         <v>3.5619109999999998</v>
@@ -7285,7 +7296,7 @@
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="51"/>
       <c r="B6" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C6" s="1">
         <v>0.63656639999999998</v>
@@ -7312,10 +7323,10 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="49" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C7" s="36">
         <v>-0.67962469999999997</v>
@@ -7353,7 +7364,7 @@
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="50"/>
       <c r="B8" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C8" s="39">
         <v>-0.8024289</v>
@@ -7391,7 +7402,7 @@
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="50"/>
       <c r="B9" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C9" s="39">
         <v>-11.448639999999999</v>
@@ -7429,7 +7440,7 @@
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="51"/>
       <c r="B10" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C10" s="41">
         <v>-10.27468</v>
@@ -7469,7 +7480,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C11" s="1">
         <v>0.27505610000000003</v>
@@ -7507,7 +7518,7 @@
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="50"/>
       <c r="B12" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C12" s="1">
         <v>0.19852059999999999</v>
@@ -7545,7 +7556,7 @@
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="50"/>
       <c r="B13" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C13" s="1">
         <v>-3.3437139999999997E-2</v>
@@ -7583,7 +7594,7 @@
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="51"/>
       <c r="B14" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C14" s="1">
         <v>-7.4605980000000002E-2</v>
@@ -7620,10 +7631,10 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="49" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C15" s="1">
         <v>0.25910539999999999</v>
@@ -7661,7 +7672,7 @@
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="50"/>
       <c r="B16" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C16" s="1">
         <v>0.1893232</v>
@@ -7699,7 +7710,7 @@
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="50"/>
       <c r="B17" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C17" s="1">
         <v>-3.3733069999999997E-2</v>
@@ -7737,7 +7748,7 @@
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="51"/>
       <c r="B18" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C18" s="1">
         <v>-7.235192E-2</v>
@@ -7777,7 +7788,7 @@
         <v>12</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C19" s="45">
         <v>0.16267690000000001</v>
@@ -7815,7 +7826,7 @@
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="50"/>
       <c r="B20" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C20" s="45">
         <v>0.1318241</v>
@@ -7853,7 +7864,7 @@
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="50"/>
       <c r="B21" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C21" s="45">
         <v>-7.6752669999999995E-2</v>
@@ -7891,7 +7902,7 @@
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="51"/>
       <c r="B22" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C22" s="45">
         <v>-6.6752569999999997E-2</v>
@@ -7922,7 +7933,7 @@
         <v>-5.0076210000000003</v>
       </c>
       <c r="M22" s="45" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="N22" s="1"/>
     </row>
@@ -7931,7 +7942,7 @@
         <v>13</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C23" s="1">
         <v>0.26141530000000002</v>
@@ -7969,7 +7980,7 @@
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="50"/>
       <c r="B24" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C24" s="1">
         <v>0.16795750000000001</v>
@@ -8007,7 +8018,7 @@
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="50"/>
       <c r="B25" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C25" s="1">
         <v>2.4449390000000001E-2</v>
@@ -8045,7 +8056,7 @@
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="51"/>
       <c r="B26" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C26" s="1">
         <v>-2.5180310000000001E-2</v>
@@ -8085,7 +8096,7 @@
         <v>14</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C27" s="1">
         <v>0.16815289999999999</v>
@@ -8123,7 +8134,7 @@
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="50"/>
       <c r="B28" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C28" s="1">
         <v>0.1095054</v>
@@ -8161,7 +8172,7 @@
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="50"/>
       <c r="B29" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C29" s="1">
         <v>4.9169679999999999E-3</v>
@@ -8199,7 +8210,7 @@
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="51"/>
       <c r="B30" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C30" s="1">
         <v>-2.9254499999999999E-2</v>
@@ -8239,7 +8250,7 @@
         <v>15</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C31" s="1">
         <v>0.10404770000000001</v>
@@ -8273,13 +8284,13 @@
         <v>3.439386E-3</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="50"/>
       <c r="B32" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C32" s="1">
         <v>3.6833039999999997E-2</v>
@@ -8313,13 +8324,13 @@
         <v>5.8418710000000002E-8</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="50"/>
       <c r="B33" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C33" s="1">
         <v>0.1045321</v>
@@ -8353,13 +8364,13 @@
         <v>3.9456639999999998E-7</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="51"/>
       <c r="B34" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C34" s="1">
         <v>3.843543E-2</v>
@@ -8393,7 +8404,7 @@
         <v>7.9669659999999998E-7</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
@@ -8401,7 +8412,7 @@
         <v>16</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C35" s="1">
         <v>-9.9169900000000005E-2</v>
@@ -8435,13 +8446,13 @@
         <v>2.0194479999999999E-4</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="50"/>
       <c r="B36" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C36" s="1">
         <v>-5.779488E-2</v>
@@ -8475,13 +8486,13 @@
         <v>1.3548390000000001E-7</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="50"/>
       <c r="B37" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C37" s="1">
         <v>-4.2352229999999998E-2</v>
@@ -8515,13 +8526,13 @@
         <v>4.2635360000000001E-3</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="51"/>
       <c r="B38" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C38" s="1">
         <v>7.5999539999999999E-3</v>
@@ -8555,7 +8566,7 @@
         <v>1.895906E-5</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
@@ -8563,7 +8574,7 @@
         <v>17</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C39" s="1">
         <v>3.6476649999999999E-2</v>
@@ -8601,7 +8612,7 @@
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" s="50"/>
       <c r="B40" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C40" s="1">
         <v>2.235734E-2</v>
@@ -8639,7 +8650,7 @@
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" s="50"/>
       <c r="B41" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C41" s="1">
         <v>4.6180759999999996E-3</v>
@@ -8677,7 +8688,7 @@
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="51"/>
       <c r="B42" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C42" s="1">
         <v>-8.7482029999999995E-3</v>
@@ -8714,13 +8725,13 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="49" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C43" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D43" s="52"/>
       <c r="E43" s="52"/>
@@ -8747,7 +8758,7 @@
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="50"/>
       <c r="B44" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C44" s="52"/>
       <c r="D44" s="52"/>
@@ -8775,7 +8786,7 @@
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="50"/>
       <c r="B45" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C45" s="52"/>
       <c r="D45" s="52"/>
@@ -8803,7 +8814,7 @@
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="51"/>
       <c r="B46" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C46" s="52"/>
       <c r="D46" s="52"/>
@@ -8830,13 +8841,13 @@
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="49" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C47" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D47" s="52"/>
       <c r="E47" s="52"/>
@@ -8863,7 +8874,7 @@
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="50"/>
       <c r="B48" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C48" s="52"/>
       <c r="D48" s="52"/>
@@ -8891,7 +8902,7 @@
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="50"/>
       <c r="B49" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C49" s="52"/>
       <c r="D49" s="52"/>
@@ -8919,7 +8930,7 @@
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="51"/>
       <c r="B50" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C50" s="52"/>
       <c r="D50" s="52"/>
@@ -8946,10 +8957,10 @@
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="49" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C51" s="45">
         <v>-4.1460160000000004</v>
@@ -8968,7 +8979,7 @@
       </c>
       <c r="H51" s="1"/>
       <c r="I51" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J51" s="52"/>
       <c r="K51" s="52"/>
@@ -8979,7 +8990,7 @@
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="50"/>
       <c r="B52" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C52" s="45">
         <v>-5.1080050000000004</v>
@@ -9007,7 +9018,7 @@
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="50"/>
       <c r="B53" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C53" s="45">
         <v>-3.7989480000000002</v>
@@ -9035,7 +9046,7 @@
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="51"/>
       <c r="B54" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C54" s="45">
         <v>-4.4755320000000003</v>
@@ -9062,10 +9073,10 @@
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="49" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C55" s="47">
         <v>0.142703</v>
@@ -9084,7 +9095,7 @@
       </c>
       <c r="H55" s="1"/>
       <c r="I55" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J55" s="52"/>
       <c r="K55" s="52"/>
@@ -9095,7 +9106,7 @@
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="50"/>
       <c r="B56" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C56" s="47">
         <v>0.10728550000000001</v>
@@ -9123,7 +9134,7 @@
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" s="50"/>
       <c r="B57" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C57" s="47">
         <v>-0.1020605</v>
@@ -9151,7 +9162,7 @@
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" s="51"/>
       <c r="B58" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C58" s="47">
         <v>-8.9823520000000004E-2</v>
@@ -9178,10 +9189,10 @@
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" s="49" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C59" s="47">
         <v>0.3732317</v>
@@ -9200,7 +9211,7 @@
       </c>
       <c r="H59" s="1"/>
       <c r="I59" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J59" s="52"/>
       <c r="K59" s="52"/>
@@ -9211,7 +9222,7 @@
     <row r="60" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A60" s="50"/>
       <c r="B60" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C60" s="47">
         <v>0.39719009999999999</v>
@@ -9239,7 +9250,7 @@
     <row r="61" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" s="50"/>
       <c r="B61" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C61" s="47">
         <v>-2.5815100000000001E-2</v>
@@ -9267,7 +9278,7 @@
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62" s="51"/>
       <c r="B62" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C62" s="47">
         <v>2.8353639999999999E-2</v>
@@ -9294,13 +9305,13 @@
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A63" s="49" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C63" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D63" s="52"/>
       <c r="E63" s="52"/>
@@ -9327,7 +9338,7 @@
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="50"/>
       <c r="B64" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C64" s="52"/>
       <c r="D64" s="52"/>
@@ -9355,7 +9366,7 @@
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="50"/>
       <c r="B65" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C65" s="52"/>
       <c r="D65" s="52"/>
@@ -9383,7 +9394,7 @@
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="51"/>
       <c r="B66" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C66" s="52"/>
       <c r="D66" s="52"/>
@@ -9410,10 +9421,10 @@
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A67" s="49" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C67" s="47">
         <v>0.2325074</v>
@@ -9432,7 +9443,7 @@
       </c>
       <c r="H67" s="1"/>
       <c r="I67" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J67" s="52"/>
       <c r="K67" s="52"/>
@@ -9443,7 +9454,7 @@
     <row r="68" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" s="50"/>
       <c r="B68" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C68" s="47">
         <v>0.28619260000000002</v>
@@ -9471,7 +9482,7 @@
     <row r="69" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A69" s="50"/>
       <c r="B69" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C69" s="47">
         <v>8.0073980000000003E-2</v>
@@ -9499,7 +9510,7 @@
     <row r="70" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70" s="51"/>
       <c r="B70" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C70" s="47">
         <v>0.1221365</v>
@@ -9526,13 +9537,13 @@
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A71" s="49" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C71" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D71" s="52"/>
       <c r="E71" s="52"/>
@@ -9559,7 +9570,7 @@
     <row r="72" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" s="50"/>
       <c r="B72" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C72" s="52"/>
       <c r="D72" s="52"/>
@@ -9587,7 +9598,7 @@
     <row r="73" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73" s="50"/>
       <c r="B73" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C73" s="52"/>
       <c r="D73" s="52"/>
@@ -9615,7 +9626,7 @@
     <row r="74" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A74" s="51"/>
       <c r="B74" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C74" s="52"/>
       <c r="D74" s="52"/>
@@ -9642,13 +9653,13 @@
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A75" s="49" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C75" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D75" s="52"/>
       <c r="E75" s="52"/>
@@ -9675,7 +9686,7 @@
     <row r="76" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A76" s="50"/>
       <c r="B76" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C76" s="52"/>
       <c r="D76" s="52"/>
@@ -9703,7 +9714,7 @@
     <row r="77" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A77" s="50"/>
       <c r="B77" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C77" s="52"/>
       <c r="D77" s="52"/>
@@ -9731,7 +9742,7 @@
     <row r="78" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A78" s="51"/>
       <c r="B78" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C78" s="52"/>
       <c r="D78" s="52"/>
@@ -9761,7 +9772,7 @@
         <v>24</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C79" s="1">
         <v>-0.9841491</v>
@@ -9780,7 +9791,7 @@
       </c>
       <c r="H79" s="1"/>
       <c r="I79" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J79" s="52"/>
       <c r="K79" s="52"/>
@@ -9791,7 +9802,7 @@
     <row r="80" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A80" s="50"/>
       <c r="B80" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C80" s="1">
         <v>0.17573549999999999</v>
@@ -9819,7 +9830,7 @@
     <row r="81" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A81" s="50"/>
       <c r="B81" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C81" s="1">
         <v>-1.1202160000000001</v>
@@ -9847,7 +9858,7 @@
     <row r="82" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A82" s="51"/>
       <c r="B82" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C82" s="1">
         <v>0.14184459999999999</v>
@@ -9877,7 +9888,7 @@
         <v>20</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C83" s="1">
         <v>1.6038840000000001</v>
@@ -9896,7 +9907,7 @@
       </c>
       <c r="H83" s="1"/>
       <c r="I83" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J83" s="52"/>
       <c r="K83" s="52"/>
@@ -9907,7 +9918,7 @@
     <row r="84" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A84" s="50"/>
       <c r="B84" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C84" s="1">
         <v>2.5716009999999998</v>
@@ -9935,7 +9946,7 @@
     <row r="85" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A85" s="50"/>
       <c r="B85" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C85" s="1">
         <v>0.61386540000000001</v>
@@ -9963,7 +9974,7 @@
     <row r="86" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A86" s="51"/>
       <c r="B86" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C86" s="1">
         <v>1.3966069999999999</v>
@@ -9993,7 +10004,7 @@
         <v>21</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C87" s="1">
         <v>16.64274</v>
@@ -10012,7 +10023,7 @@
       </c>
       <c r="H87" s="1"/>
       <c r="I87" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J87" s="52"/>
       <c r="K87" s="52"/>
@@ -10023,7 +10034,7 @@
     <row r="88" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A88" s="50"/>
       <c r="B88" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C88" s="1">
         <v>19.986529999999998</v>
@@ -10051,7 +10062,7 @@
     <row r="89" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A89" s="50"/>
       <c r="B89" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C89" s="1">
         <v>-4.4803540000000002</v>
@@ -10079,7 +10090,7 @@
     <row r="90" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A90" s="51"/>
       <c r="B90" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C90" s="1">
         <v>-0.82880399999999999</v>
@@ -10105,30 +10116,30 @@
       <c r="N90" s="1"/>
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A91" s="49" t="s">
-        <v>25</v>
+      <c r="A91" s="70" t="s">
+        <v>151</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C91" s="1">
-        <v>0.28573979999999999</v>
-      </c>
-      <c r="D91" s="1">
-        <v>2.892964E-2</v>
-      </c>
-      <c r="E91" s="1">
-        <v>20.899597</v>
-      </c>
-      <c r="F91" s="1">
-        <v>9.8770609999999994</v>
-      </c>
-      <c r="G91" s="2">
-        <v>2.5221599999999999E-9</v>
+        <v>106</v>
+      </c>
+      <c r="C91" s="45">
+        <v>264.8</v>
+      </c>
+      <c r="D91" s="45">
+        <v>32.234110000000001</v>
+      </c>
+      <c r="E91" s="45">
+        <v>30.811264000000001</v>
+      </c>
+      <c r="F91" s="45">
+        <v>8.2149009999999993</v>
+      </c>
+      <c r="G91" s="45">
+        <v>2.9384279999999999E-9</v>
       </c>
       <c r="H91" s="1"/>
       <c r="I91" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J91" s="52"/>
       <c r="K91" s="52"/>
@@ -10137,24 +10148,24 @@
       <c r="N91" s="1"/>
     </row>
     <row r="92" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A92" s="50"/>
+      <c r="A92" s="71"/>
       <c r="B92" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="C92" s="1">
-        <v>0.38685409999999998</v>
-      </c>
-      <c r="D92" s="1">
-        <v>2.990483E-2</v>
-      </c>
-      <c r="E92" s="1">
-        <v>24.614989999999999</v>
-      </c>
-      <c r="F92" s="1">
-        <v>12.936170000000001</v>
-      </c>
-      <c r="G92" s="2">
-        <v>1.7821690000000001E-12</v>
+        <v>107</v>
+      </c>
+      <c r="C92" s="45">
+        <v>249.71430000000001</v>
+      </c>
+      <c r="D92" s="45">
+        <v>24.47692</v>
+      </c>
+      <c r="E92" s="45">
+        <v>40.626759999999997</v>
+      </c>
+      <c r="F92" s="45">
+        <v>10.202030000000001</v>
+      </c>
+      <c r="G92" s="45">
+        <v>9.0369680000000005E-13</v>
       </c>
       <c r="H92" s="1"/>
       <c r="I92" s="52"/>
@@ -10165,24 +10176,24 @@
       <c r="N92" s="1"/>
     </row>
     <row r="93" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A93" s="50"/>
+      <c r="A93" s="71"/>
       <c r="B93" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C93" s="1">
-        <v>2.0270739999999999E-2</v>
-      </c>
-      <c r="D93" s="1">
-        <v>2.7636999999999998E-2</v>
-      </c>
-      <c r="E93" s="1">
-        <v>40</v>
-      </c>
-      <c r="F93" s="1">
-        <v>0.733464</v>
-      </c>
-      <c r="G93" s="1">
-        <v>0.46755279999999999</v>
+        <v>108</v>
+      </c>
+      <c r="C93" s="45">
+        <v>43.209679999999999</v>
+      </c>
+      <c r="D93" s="45">
+        <v>56.537500000000001</v>
+      </c>
+      <c r="E93" s="45">
+        <v>16.96773</v>
+      </c>
+      <c r="F93" s="45">
+        <v>0.7642658</v>
+      </c>
+      <c r="G93" s="45">
+        <v>0.45520664523399601</v>
       </c>
       <c r="H93" s="1"/>
       <c r="I93" s="52"/>
@@ -10193,24 +10204,24 @@
       <c r="N93" s="1"/>
     </row>
     <row r="94" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A94" s="51"/>
+      <c r="A94" s="72"/>
       <c r="B94" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="C94" s="1">
-        <v>0.13333100000000001</v>
-      </c>
-      <c r="D94" s="1">
-        <v>5.6024570000000003E-2</v>
-      </c>
-      <c r="E94" s="1">
-        <v>8.8358460000000001</v>
-      </c>
-      <c r="F94" s="1">
-        <v>2.3798659999999998</v>
-      </c>
-      <c r="G94" s="2">
-        <v>4.1726619999999999E-2</v>
+        <v>109</v>
+      </c>
+      <c r="C94" s="45">
+        <v>32.259779999999999</v>
+      </c>
+      <c r="D94" s="45">
+        <v>15.415459999999999</v>
+      </c>
+      <c r="E94" s="45">
+        <v>17.28622</v>
+      </c>
+      <c r="F94" s="45">
+        <v>2.0926900000000002</v>
+      </c>
+      <c r="G94" s="45">
+        <v>5.14251187538E-2</v>
       </c>
       <c r="H94" s="1"/>
       <c r="I94" s="52"/>
@@ -10222,10 +10233,10 @@
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A95" s="49" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C95" s="1">
         <v>1.3623919999999999E-2</v>
@@ -10244,7 +10255,7 @@
       </c>
       <c r="H95" s="1"/>
       <c r="I95" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J95" s="52"/>
       <c r="K95" s="52"/>
@@ -10255,7 +10266,7 @@
     <row r="96" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A96" s="50"/>
       <c r="B96" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C96" s="1">
         <v>7.6710570000000006E-2</v>
@@ -10283,7 +10294,7 @@
     <row r="97" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A97" s="50"/>
       <c r="B97" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C97" s="1">
         <v>-6.9491259999999999E-2</v>
@@ -10311,7 +10322,7 @@
     <row r="98" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A98" s="51"/>
       <c r="B98" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C98" s="1">
         <v>-6.8129929999999998E-3</v>
@@ -10338,10 +10349,10 @@
     </row>
     <row r="99" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A99" s="49" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C99" s="45">
         <v>2.012891E-5</v>
@@ -10360,7 +10371,7 @@
       </c>
       <c r="H99" s="1"/>
       <c r="I99" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J99" s="52"/>
       <c r="K99" s="52"/>
@@ -10371,7 +10382,7 @@
     <row r="100" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A100" s="50"/>
       <c r="B100" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C100" s="45">
         <v>8.7200299999999999E-4</v>
@@ -10399,7 +10410,7 @@
     <row r="101" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A101" s="50"/>
       <c r="B101" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C101" s="45">
         <v>-2.0367390000000001E-3</v>
@@ -10427,7 +10438,7 @@
     <row r="102" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A102" s="51"/>
       <c r="B102" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C102" s="45">
         <v>-1.576327E-3</v>
@@ -10453,30 +10464,30 @@
       <c r="N102" s="1"/>
     </row>
     <row r="103" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A103" s="49" t="s">
-        <v>26</v>
+      <c r="A103" s="70" t="s">
+        <v>25</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C103" s="1">
-        <v>0.29603849999999998</v>
+        <v>0.29653109999999999</v>
       </c>
       <c r="D103" s="1">
-        <v>3.2874760000000003E-2</v>
+        <v>3.0081920000000002E-2</v>
       </c>
       <c r="E103" s="1">
-        <v>18.839901000000001</v>
+        <v>12.984576000000001</v>
       </c>
       <c r="F103" s="1">
-        <v>9.0050399999999993</v>
+        <v>9.8574540000000006</v>
       </c>
       <c r="G103" s="2">
-        <v>2.974355E-8</v>
+        <v>2.1465810000000001E-7</v>
       </c>
       <c r="H103" s="1"/>
       <c r="I103" s="52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J103" s="52"/>
       <c r="K103" s="52"/>
@@ -10485,24 +10496,24 @@
       <c r="N103" s="1"/>
     </row>
     <row r="104" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A104" s="50"/>
+      <c r="A104" s="71"/>
       <c r="B104" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C104" s="1">
-        <v>0.48750929999999998</v>
+        <v>0.48443409999999998</v>
       </c>
       <c r="D104" s="1">
-        <v>2.0179229999999999E-2</v>
+        <v>1.925058E-2</v>
       </c>
       <c r="E104" s="1">
-        <v>33.068705000000001</v>
+        <v>33.275270999999996</v>
       </c>
       <c r="F104" s="1">
-        <v>24.15896</v>
+        <v>25.164650000000002</v>
       </c>
       <c r="G104" s="2">
-        <v>1.3818109999999999E-22</v>
+        <v>3.0964249999999998E-23</v>
       </c>
       <c r="H104" s="1"/>
       <c r="I104" s="52"/>
@@ -10513,24 +10524,24 @@
       <c r="N104" s="1"/>
     </row>
     <row r="105" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A105" s="50"/>
+      <c r="A105" s="71"/>
       <c r="B105" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C105" s="1">
-        <v>-4.929849E-2</v>
+        <v>-4.9176770000000002E-2</v>
       </c>
       <c r="D105" s="1">
-        <v>3.1121630000000001E-2</v>
+        <v>3.2182200000000001E-2</v>
       </c>
       <c r="E105" s="1">
-        <v>4.2666779999999997</v>
+        <v>6.754302</v>
       </c>
       <c r="F105" s="1">
-        <v>-1.5840590000000001</v>
+        <v>-1.5280739999999999</v>
       </c>
       <c r="G105" s="1">
-        <v>0.18392030000000001</v>
+        <v>0.17187649999999999</v>
       </c>
       <c r="H105" s="1"/>
       <c r="I105" s="52"/>
@@ -10541,24 +10552,24 @@
       <c r="N105" s="1"/>
     </row>
     <row r="106" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A106" s="51"/>
+      <c r="A106" s="72"/>
       <c r="B106" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C106" s="1">
-        <v>0.15619479999999999</v>
+        <v>0.14682600000000001</v>
       </c>
       <c r="D106" s="1">
-        <v>2.6369159999999999E-2</v>
+        <v>2.4250879999999999E-2</v>
       </c>
       <c r="E106" s="1">
-        <v>5.0675150000000002</v>
+        <v>6.7890449999999998</v>
       </c>
       <c r="F106" s="1">
-        <v>5.9233900000000004</v>
+        <v>6.0544589999999996</v>
       </c>
       <c r="G106" s="2">
-        <v>1.86768E-3</v>
+        <v>5.7776140000000001E-4</v>
       </c>
       <c r="H106" s="1"/>
       <c r="I106" s="52"/>
@@ -10588,22 +10599,20 @@
     </row>
   </sheetData>
   <mergeCells count="45">
-    <mergeCell ref="I1:N1"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="A7:A10"/>
-    <mergeCell ref="I3:M6"/>
-    <mergeCell ref="A23:A26"/>
-    <mergeCell ref="A27:A30"/>
-    <mergeCell ref="A11:A14"/>
-    <mergeCell ref="A15:A18"/>
-    <mergeCell ref="C1:H1"/>
-    <mergeCell ref="A19:A22"/>
-    <mergeCell ref="A31:A34"/>
-    <mergeCell ref="A35:A38"/>
-    <mergeCell ref="A39:A42"/>
-    <mergeCell ref="A55:A58"/>
-    <mergeCell ref="A47:A50"/>
-    <mergeCell ref="A51:A54"/>
+    <mergeCell ref="A95:A98"/>
+    <mergeCell ref="I95:M98"/>
+    <mergeCell ref="A103:A106"/>
+    <mergeCell ref="I103:M106"/>
+    <mergeCell ref="A91:A94"/>
+    <mergeCell ref="I91:M94"/>
+    <mergeCell ref="A99:A102"/>
+    <mergeCell ref="I99:M102"/>
+    <mergeCell ref="A87:A90"/>
+    <mergeCell ref="I87:M90"/>
+    <mergeCell ref="A75:A78"/>
+    <mergeCell ref="C75:G78"/>
+    <mergeCell ref="A79:A82"/>
+    <mergeCell ref="I79:M82"/>
     <mergeCell ref="C47:G50"/>
     <mergeCell ref="A43:A46"/>
     <mergeCell ref="C43:G46"/>
@@ -10619,20 +10628,22 @@
     <mergeCell ref="C63:G66"/>
     <mergeCell ref="A59:A62"/>
     <mergeCell ref="I59:M62"/>
-    <mergeCell ref="A87:A90"/>
-    <mergeCell ref="I87:M90"/>
-    <mergeCell ref="A75:A78"/>
-    <mergeCell ref="C75:G78"/>
-    <mergeCell ref="A79:A82"/>
-    <mergeCell ref="I79:M82"/>
-    <mergeCell ref="A95:A98"/>
-    <mergeCell ref="I95:M98"/>
-    <mergeCell ref="A103:A106"/>
-    <mergeCell ref="I103:M106"/>
-    <mergeCell ref="A91:A94"/>
-    <mergeCell ref="I91:M94"/>
-    <mergeCell ref="A99:A102"/>
-    <mergeCell ref="I99:M102"/>
+    <mergeCell ref="A31:A34"/>
+    <mergeCell ref="A35:A38"/>
+    <mergeCell ref="A39:A42"/>
+    <mergeCell ref="A55:A58"/>
+    <mergeCell ref="A47:A50"/>
+    <mergeCell ref="A51:A54"/>
+    <mergeCell ref="A27:A30"/>
+    <mergeCell ref="A11:A14"/>
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="C1:H1"/>
+    <mergeCell ref="A19:A22"/>
+    <mergeCell ref="I1:N1"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="A7:A10"/>
+    <mergeCell ref="I3:M6"/>
+    <mergeCell ref="A23:A26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>